<commit_message>
feat: update PDF conversion message for batch processing
</commit_message>
<xml_diff>
--- a/input/02_input_spp.xlsx
+++ b/input/02_input_spp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Documents\repo\latsar\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A1345F-80CB-44E7-BEB2-08E79C9B963B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D871F2-6463-4589-94DE-C8B858DA5057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_mitra" sheetId="1" r:id="rId1"/>
@@ -161,7 +161,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -190,6 +190,12 @@
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -211,13 +217,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,79 +464,79 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="6" t="s">
         <v>38</v>
       </c>
     </row>
@@ -643,79 +651,79 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="6" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="6" t="s">
         <v>40</v>
       </c>
     </row>
@@ -755,104 +763,104 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="6">
         <v>585</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="6">
         <v>254</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="7">
         <v>50.5550193050193</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="6">
         <v>408</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="6">
         <v>180</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="7">
         <v>47.477982385908732</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="6">
         <v>390</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="6">
         <v>187</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="7">
         <v>47.477982385908732</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="6">
         <v>362</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="6">
         <v>164</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="7">
         <v>47.477982385908732</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="6">
         <v>376</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="6">
         <v>172</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="7">
         <v>45.744680851063826</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="6">
         <v>377</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="6">
         <v>196</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="7">
         <v>51.989389920424401</v>
       </c>
     </row>

</xml_diff>